<commit_message>
docs: update prompts report and controllers
</commit_message>
<xml_diff>
--- a/чек-лист.xlsx
+++ b/чек-лист.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Huawei\Desktop\architect_ivan_var_8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03B60FFD-A720-49FF-BE51-561AC0B33763}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AFC2BE1-6F18-41A4-BA06-BF50E6F8CC80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="11520" windowHeight="13800" xr2:uid="{4D2451AB-8DE5-4CF7-9623-478264A7A8F6}"/>
   </bookViews>
@@ -842,7 +842,7 @@
       </c>
       <c r="D1" s="9">
         <f>SUM(чек_лист[Column1])</f>
-        <v>97</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1473,11 +1473,11 @@
         <v>6</v>
       </c>
       <c r="D37" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37">
         <f>чек_лист[[#This Row],[Выполнение (1 или 0) ЗАПОЛНЯЕМ]]*чек_лист[[#This Row],[Баллы (0-2)]]</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
@@ -1491,11 +1491,11 @@
         <v>6</v>
       </c>
       <c r="D38" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38">
         <f>чек_лист[[#This Row],[Выполнение (1 или 0) ЗАПОЛНЯЕМ]]*чек_лист[[#This Row],[Баллы (0-2)]]</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -1509,11 +1509,11 @@
         <v>6</v>
       </c>
       <c r="D39" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39">
         <f>чек_лист[[#This Row],[Выполнение (1 или 0) ЗАПОЛНЯЕМ]]*чек_лист[[#This Row],[Баллы (0-2)]]</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -2013,11 +2013,11 @@
         <v>18</v>
       </c>
       <c r="D67" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E67">
         <f>чек_лист[[#This Row],[Выполнение (1 или 0) ЗАПОЛНЯЕМ]]*чек_лист[[#This Row],[Баллы (0-2)]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
@@ -2031,11 +2031,11 @@
         <v>18</v>
       </c>
       <c r="D68" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E68">
         <f>чек_лист[[#This Row],[Выполнение (1 или 0) ЗАПОЛНЯЕМ]]*чек_лист[[#This Row],[Баллы (0-2)]]</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">

</xml_diff>